<commit_message>
ajout de la page UFC
</commit_message>
<xml_diff>
--- a/fiche_de_calcul.xlsx
+++ b/fiche_de_calcul.xlsx
@@ -5,12 +5,13 @@
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="Halstead" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="LOC" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="CC" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="UFC" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="62" uniqueCount="52">
   <si>
     <t xml:space="preserve">Opérateurs</t>
   </si>
@@ -174,6 +175,62 @@
     <t xml:space="preserve">Calcul : 
 (CC = [E – N] +2)</t>
   </si>
+  <si>
+    <t xml:space="preserve">Tableau des poids</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Catégorie</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Simple</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moyen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difficile</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entrées externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sorties externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Requete externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers internes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fichiers externes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tableau des scores</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Formule UFC score :
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(use de SOMMEPROD) </t>
+    </r>
+  </si>
 </sst>
 </file>
 
@@ -182,7 +239,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="General"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -204,12 +261,6 @@
       <sz val="10"/>
       <name val="Arial"/>
       <family val="0"/>
-    </font>
-    <font>
-      <sz val="12"/>
-      <color theme="1"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
     </font>
     <font>
       <i val="true"/>
@@ -247,6 +298,26 @@
       <color theme="1"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -313,61 +384,85 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -390,37 +485,37 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="FFFFFF"/>
+        <a:srgbClr val="ffffff"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="0E2841"/>
+        <a:srgbClr val="0e2841"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="E8E8E8"/>
+        <a:srgbClr val="e8e8e8"/>
       </a:lt2>
       <a:accent1>
         <a:srgbClr val="156082"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="E97132"/>
+        <a:srgbClr val="e97132"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="196B24"/>
+        <a:srgbClr val="196b24"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="0F9ED5"/>
+        <a:srgbClr val="0f9ed5"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="A02B93"/>
+        <a:srgbClr val="a02b93"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="4EA72E"/>
+        <a:srgbClr val="4ea72e"/>
       </a:accent6>
       <a:hlink>
         <a:srgbClr val="467886"/>
       </a:hlink>
       <a:folHlink>
-        <a:srgbClr val="96607D"/>
+        <a:srgbClr val="96607d"/>
       </a:folHlink>
     </a:clrScheme>
     <a:fontScheme name="Office">
@@ -562,164 +657,164 @@
   <dimension ref="A1:E22"/>
   <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.34"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="33.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="33.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="1" t="s">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="D3" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="1" t="s">
+      <c r="A4" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="1" t="s">
+      <c r="A5" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="2" t="s">
+      <c r="D5" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="1" t="s">
+      <c r="A6" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="2" t="n">
+      <c r="D6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="0" t="n">
+      <c r="E6" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="1" t="s">
+      <c r="A7" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="2" t="n">
+      <c r="D7" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="1" t="s">
+      <c r="A8" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="1" t="s">
+      <c r="A9" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="2" t="s">
+      <c r="D9" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="1" t="s">
+      <c r="A10" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="1" t="s">
+      <c r="A11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3" t="s">
+      <c r="A12" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="2" t="n">
+      <c r="B12" s="3" t="n">
         <f aca="false">SUM(B2:B11)</f>
         <v>16</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="4" t="n">
+      <c r="D12" s="3" t="n">
         <f aca="false">ROWS(D2:D9)</f>
         <v>8</v>
       </c>
@@ -728,83 +823,84 @@
       <c r="A13" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="0" t="s">
+      <c r="C13" s="1" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+      <c r="A14" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="2" t="n">
+      <c r="B14" s="3" t="n">
         <f aca="false">ROWS(B2:B11)</f>
         <v>10</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="2" t="n">
+      <c r="D14" s="3" t="n">
         <f aca="false">SUM(E2:E9)</f>
         <v>35</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <f aca="false">B12+D14</f>
         <v>51</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <f aca="false">B14+D12</f>
         <v>18</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <f aca="false">B18*LOG(B19,2)</f>
         <v>212.666175073558</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <f aca="false">(B14/2)*(D14/D12)</f>
         <v>21.875</v>
       </c>
     </row>
-    <row r="22" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <f aca="false">B21*B20</f>
         <v>4652.07257973408</v>
       </c>
@@ -829,10 +925,10 @@
   <sheetFormatPr defaultColWidth="10.4609375" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="6" t="n">
+      <c r="B1" s="2" t="n">
         <v>920</v>
       </c>
     </row>
@@ -855,318 +951,318 @@
   <dimension ref="A1:G33"/>
   <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="6" width="23.81"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="6" width="13.08"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="23.81"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="13.08"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="8" t="s">
+      <c r="B1" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="9" t="s">
+      <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="10" t="n">
+      <c r="B2" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="11" t="s">
+      <c r="A3" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="10" t="n">
+      <c r="B3" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="10" t="n">
+      <c r="B4" s="9" t="n">
         <f aca="false">B3 - B2 + 2</f>
         <v>4</v>
       </c>
-      <c r="C4" s="10"/>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10"/>
-      <c r="G4" s="10"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="13"/>
-      <c r="B6" s="10"/>
-      <c r="C6" s="10"/>
-      <c r="D6" s="10"/>
-      <c r="E6" s="10"/>
-      <c r="F6" s="10"/>
-      <c r="G6" s="10"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13"/>
-      <c r="B7" s="10"/>
-      <c r="C7" s="10"/>
-      <c r="D7" s="10"/>
-      <c r="E7" s="10"/>
-      <c r="F7" s="10"/>
-      <c r="G7" s="10"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="13"/>
-      <c r="B8" s="10"/>
-      <c r="C8" s="10"/>
-      <c r="D8" s="10"/>
-      <c r="E8" s="10"/>
-      <c r="F8" s="10"/>
-      <c r="G8" s="10"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="13"/>
-      <c r="B9" s="10"/>
-      <c r="C9" s="10"/>
-      <c r="D9" s="10"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="10"/>
-      <c r="G9" s="10"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13"/>
-      <c r="B10" s="10"/>
-      <c r="C10" s="10"/>
-      <c r="D10" s="10"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="10"/>
-      <c r="G10" s="10"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13"/>
-      <c r="B11" s="10"/>
-      <c r="C11" s="10"/>
-      <c r="D11" s="10"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="10"/>
-      <c r="G11" s="10"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="13"/>
-      <c r="B12" s="10"/>
-      <c r="C12" s="10"/>
-      <c r="D12" s="10"/>
-      <c r="E12" s="10"/>
-      <c r="F12" s="10"/>
-      <c r="G12" s="10"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="13"/>
-      <c r="B13" s="10"/>
-      <c r="C13" s="10"/>
-      <c r="D13" s="10"/>
-      <c r="E13" s="10"/>
-      <c r="F13" s="10"/>
-      <c r="G13" s="10"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="13"/>
-      <c r="B14" s="10"/>
-      <c r="C14" s="10"/>
-      <c r="D14" s="10"/>
-      <c r="E14" s="10"/>
-      <c r="F14" s="10"/>
-      <c r="G14" s="10"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13"/>
-      <c r="B15" s="10"/>
-      <c r="C15" s="10"/>
-      <c r="D15" s="10"/>
-      <c r="E15" s="10"/>
-      <c r="F15" s="10"/>
-      <c r="G15" s="10"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13"/>
-      <c r="B16" s="10"/>
-      <c r="C16" s="10"/>
-      <c r="D16" s="10"/>
-      <c r="E16" s="10"/>
-      <c r="F16" s="10"/>
-      <c r="G16" s="10"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13"/>
-      <c r="B17" s="10"/>
-      <c r="C17" s="10"/>
-      <c r="D17" s="10"/>
-      <c r="E17" s="10"/>
-      <c r="F17" s="10"/>
-      <c r="G17" s="10"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="13"/>
-      <c r="B18" s="10"/>
-      <c r="C18" s="10"/>
-      <c r="D18" s="10"/>
-      <c r="E18" s="10"/>
-      <c r="F18" s="10"/>
-      <c r="G18" s="10"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="13"/>
-      <c r="B19" s="10"/>
-      <c r="C19" s="10"/>
-      <c r="D19" s="10"/>
-      <c r="E19" s="10"/>
-      <c r="F19" s="10"/>
-      <c r="G19" s="10"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="13"/>
-      <c r="B20" s="10"/>
-      <c r="C20" s="10"/>
-      <c r="D20" s="10"/>
-      <c r="E20" s="10"/>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13"/>
-      <c r="B21" s="10"/>
-      <c r="C21" s="10"/>
-      <c r="D21" s="10"/>
-      <c r="E21" s="10"/>
-      <c r="F21" s="10"/>
-      <c r="G21" s="10"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="10"/>
-      <c r="B22" s="10"/>
-      <c r="C22" s="10"/>
-      <c r="D22" s="10"/>
-      <c r="E22" s="10"/>
-      <c r="F22" s="10"/>
-      <c r="G22" s="10"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="10"/>
-      <c r="B23" s="10"/>
-      <c r="C23" s="10"/>
-      <c r="D23" s="10"/>
-      <c r="E23" s="10"/>
-      <c r="F23" s="10"/>
-      <c r="G23" s="10"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="10"/>
-      <c r="B24" s="10"/>
-      <c r="C24" s="10"/>
-      <c r="D24" s="10"/>
-      <c r="E24" s="10"/>
-      <c r="F24" s="10"/>
-      <c r="G24" s="10"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="10"/>
-      <c r="B25" s="10"/>
-      <c r="C25" s="10"/>
-      <c r="D25" s="10"/>
-      <c r="E25" s="10"/>
-      <c r="F25" s="10"/>
-      <c r="G25" s="10"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="10"/>
-      <c r="B26" s="10"/>
-      <c r="C26" s="10"/>
-      <c r="D26" s="10"/>
-      <c r="E26" s="10"/>
-      <c r="F26" s="10"/>
-      <c r="G26" s="10"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="10"/>
-      <c r="B27" s="10"/>
-      <c r="C27" s="10"/>
-      <c r="D27" s="10"/>
-      <c r="E27" s="10"/>
-      <c r="F27" s="10"/>
-      <c r="G27" s="10"/>
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="10"/>
-      <c r="B28" s="10"/>
-      <c r="C28" s="10"/>
-      <c r="D28" s="10"/>
-      <c r="E28" s="10"/>
-      <c r="F28" s="10"/>
-      <c r="G28" s="10"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="10"/>
-      <c r="B29" s="10"/>
-      <c r="C29" s="10"/>
-      <c r="D29" s="10"/>
-      <c r="E29" s="10"/>
-      <c r="F29" s="10"/>
-      <c r="G29" s="10"/>
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="10"/>
-      <c r="B30" s="10"/>
-      <c r="C30" s="10"/>
-      <c r="D30" s="10"/>
-      <c r="E30" s="10"/>
-      <c r="F30" s="10"/>
-      <c r="G30" s="10"/>
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="10"/>
-      <c r="B31" s="10"/>
-      <c r="C31" s="10"/>
-      <c r="D31" s="10"/>
-      <c r="E31" s="10"/>
-      <c r="F31" s="10"/>
-      <c r="G31" s="10"/>
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="10"/>
-      <c r="B32" s="10"/>
-      <c r="C32" s="10"/>
-      <c r="D32" s="10"/>
-      <c r="E32" s="10"/>
-      <c r="F32" s="10"/>
-      <c r="G32" s="10"/>
+      <c r="A32" s="9"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="10"/>
-      <c r="B33" s="10"/>
-      <c r="C33" s="10"/>
-      <c r="D33" s="10"/>
-      <c r="E33" s="10"/>
-      <c r="F33" s="10"/>
-      <c r="G33" s="10"/>
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1177,4 +1273,228 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:D21"/>
+  <sheetFormatPr defaultColWidth="11.74609375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.74"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="35.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B1" s="13"/>
+    </row>
+    <row r="2" customFormat="false" ht="20.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B2" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C2" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D2" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="19.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C3" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D3" s="0" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B4" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C4" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D4" s="0" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="20" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B5" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="0" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="22.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C6" s="0" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="0" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="22.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="D7" s="0" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="32.65" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B10" s="13"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="14" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="C11" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="15" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="B12" s="0" t="n">
+        <v>4</v>
+      </c>
+      <c r="C12" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="D12" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="18.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="17" t="s">
+        <v>46</v>
+      </c>
+      <c r="B13" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="0" t="n">
+        <v>2</v>
+      </c>
+      <c r="D13" s="0" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="19.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="17" t="s">
+        <v>47</v>
+      </c>
+      <c r="B14" s="0" t="n">
+        <v>7</v>
+      </c>
+      <c r="C14" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="19.2" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B15" s="0" t="n">
+        <v>3</v>
+      </c>
+      <c r="C15" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="0" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="18.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="B16" s="0" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="0" t="n">
+        <v>5</v>
+      </c>
+      <c r="D16" s="0" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="8.45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="18"/>
+      <c r="B17" s="18"/>
+      <c r="C17" s="18"/>
+      <c r="D17" s="18"/>
+    </row>
+    <row r="18" customFormat="false" ht="8.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="19" customFormat="false" ht="8.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+    <row r="20" customFormat="false" ht="33.05" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B20" s="0" t="n">
+        <f aca="false">SUMPRODUCT(B3:D7,B12:D16)</f>
+        <v>144</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="27.3" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:B1"/>
+    <mergeCell ref="A10:B10"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ajout du calcul UFC de QuickSort pour la question 9
</commit_message>
<xml_diff>
--- a/fiche_de_calcul.xlsx
+++ b/fiche_de_calcul.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns2="http://schemas.libreoffice.org/">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,14 +8,15 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Halstead" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="LOC" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="CC" sheetId="3" state="visible" r:id="rId5"/>
+    <sheet name="Halstead" sheetId="1" state="visible" ns1:id="rId3"/>
+    <sheet name="LOC" sheetId="2" state="visible" ns1:id="rId4"/>
+    <sheet name="CC" sheetId="3" state="visible" ns1:id="rId5"/>
+    <sheet name="UFC QuickSort" sheetId="4" ns1:id="rIdQ9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    <ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <ns2:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -179,10 +180,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
+    <numFmt numFmtId="165" formatCode="General"/>
+    <numFmt numFmtId="166" formatCode="General"/>
+    <numFmt numFmtId="167" formatCode="0"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="33">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -249,16 +253,170 @@
       <family val="1"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+      <family val="0"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <i val="true"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="12">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -287,6 +445,45 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="false" diagonalDown="false">
+      <left/>
+      <right style="thin"/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border diagonalUp="0" diagonalDown="0"/>
+    <border diagonalUp="0" diagonalDown="0">
+      <right style="thin"/>
+      <bottom style="thin"/>
+    </border>
+    <border diagonalUp="0" diagonalDown="0">
+      <bottom style="thin"/>
+    </border>
+    <border diagonalUp="0" diagonalDown="0">
+      <right style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -313,7 +510,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="51">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -369,6 +566,131 @@
     <xf numFmtId="164" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="14" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="15" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="10" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="5" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="17" fillId="2" borderId="6" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="18" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="4" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="19" fillId="2" borderId="7" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="4" borderId="8" xfId="0" applyFont="0" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="0">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="24" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="25" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="20" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="4" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="4" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="28" fillId="4" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="4" borderId="8" xfId="0" applyFont="1" applyBorder="0" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="4" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="4" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="29" fillId="4" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="30" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="31" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="30" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="32" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="32" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="32" fillId="6" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="7" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="0"/>
+    </xf>
+    <xf numFmtId="166" fontId="30" fillId="4" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="general" vertical="bottom" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1177,4 +1499,376 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="26" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="14" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="14" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="14" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="14" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="14" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="14" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="43" t="str">
+        <v>Q9 - Points de fonction de QuickSort</v>
+      </c>
+      <c r="B1" s="42"/>
+      <c r="C1" s="42"/>
+      <c r="D1" s="42"/>
+      <c r="E1" s="42"/>
+      <c r="F1" s="42"/>
+      <c r="G1" s="42"/>
+      <c r="H1" s="42"/>
+    </row>
+    <row r="2" ht="24" customHeight="1">
+      <c r="A2" s="42"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
+      <c r="H2" s="42"/>
+    </row>
+    <row r="3" ht="24" customHeight="1">
+      <c r="A3" s="45" t="str">
+        <v>Catégorie</v>
+      </c>
+      <c r="B3" s="45" t="str">
+        <v>Poids</v>
+      </c>
+      <c r="C3" s="45"/>
+      <c r="D3" s="45"/>
+      <c r="E3" s="45" t="str">
+        <v>Scores</v>
+      </c>
+      <c r="F3" s="45"/>
+      <c r="G3" s="45"/>
+      <c r="H3" s="45" t="str">
+        <v>Total pondéré</v>
+      </c>
+    </row>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="45"/>
+      <c r="B4" s="45" t="str">
+        <v>Simple</v>
+      </c>
+      <c r="C4" s="45" t="str">
+        <v>Moyen</v>
+      </c>
+      <c r="D4" s="45" t="str">
+        <v>Difficile</v>
+      </c>
+      <c r="E4" s="45" t="str">
+        <v>Simple</v>
+      </c>
+      <c r="F4" s="45" t="str">
+        <v>Moyen</v>
+      </c>
+      <c r="G4" s="45" t="str">
+        <v>Difficile</v>
+      </c>
+      <c r="H4" s="45"/>
+    </row>
+    <row r="5" ht="24" customHeight="1">
+      <c r="A5" s="42" t="str">
+        <v>Entrées externes</v>
+      </c>
+      <c r="B5" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D5" s="47" t="n">
+        <v>6</v>
+      </c>
+      <c r="E5" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F5" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="47" t="n">
+        <f>B5*E5+C5*F5+D5*G5</f>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="24" customHeight="1">
+      <c r="A6" s="42" t="str">
+        <v>Sorties externes</v>
+      </c>
+      <c r="B6" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="D6" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="E6" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="47" t="n">
+        <f>B6*E6+C6*F6+D6*G6</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" ht="24" customHeight="1">
+      <c r="A7" s="42" t="str">
+        <v>Requêtes externes</v>
+      </c>
+      <c r="B7" s="47" t="n">
+        <v>3</v>
+      </c>
+      <c r="C7" s="47" t="n">
+        <v>4</v>
+      </c>
+      <c r="D7" s="47" t="n">
+        <v>6</v>
+      </c>
+      <c r="E7" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="47" t="n">
+        <f>B7*E7+C7*F7+D7*G7</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1">
+      <c r="A8" s="42" t="str">
+        <v>Fichiers internes</v>
+      </c>
+      <c r="B8" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="C8" s="47" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="47" t="n">
+        <v>15</v>
+      </c>
+      <c r="E8" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="47" t="n">
+        <f>B8*E8+C8*F8+D8*G8</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="24" customHeight="1">
+      <c r="A9" s="42" t="str">
+        <v>Fichiers externes</v>
+      </c>
+      <c r="B9" s="47" t="n">
+        <v>5</v>
+      </c>
+      <c r="C9" s="47" t="n">
+        <v>7</v>
+      </c>
+      <c r="D9" s="47" t="n">
+        <v>10</v>
+      </c>
+      <c r="E9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="49" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="47" t="n">
+        <f>B9*E9+C9*F9+D9*G9</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="24" customHeight="1">
+      <c r="A10" s="45" t="str">
+        <v>UFC</v>
+      </c>
+      <c r="B10" s="48"/>
+      <c r="C10" s="48"/>
+      <c r="D10" s="48"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
+      <c r="G10" s="48"/>
+      <c r="H10" s="48" t="n">
+        <f>SUM(H5:H9)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="11" ht="24" customHeight="1">
+      <c r="A11" s="42"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
+      <c r="G11" s="42"/>
+      <c r="H11" s="42"/>
+    </row>
+    <row r="12" ht="24" customHeight="1">
+      <c r="A12" s="46" t="str">
+        <v>Hypothèses et justification</v>
+      </c>
+      <c r="B12" s="42"/>
+      <c r="C12" s="42"/>
+      <c r="D12" s="42"/>
+      <c r="E12" s="42"/>
+      <c r="F12" s="42"/>
+      <c r="G12" s="42"/>
+      <c r="H12" s="42"/>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="50" t="str">
+        <v>Périmètre : adaptation pédagogique au service de tri iqsort0(a, n), appelé depuis l’extérieur.</v>
+      </c>
+      <c r="B13" s="50"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
+      <c r="F13" s="50"/>
+      <c r="G13" s="50"/>
+      <c r="H13" s="50"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="50" t="str">
+        <v>Entrée simple : une demande de tri reçoit le tableau a et sa taille n. Les deux paramètres constituent une seule entrée.</v>
+      </c>
+      <c r="B14" s="50"/>
+      <c r="C14" s="50"/>
+      <c r="D14" s="50"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="50"/>
+      <c r="G14" s="50"/>
+      <c r="H14" s="50"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="50" t="str">
+        <v>Sortie simple : le tableau trié est accessible à l’appelant après modification en place, même si la fonction est void.</v>
+      </c>
+      <c r="B15" s="50"/>
+      <c r="C15" s="50"/>
+      <c r="D15" s="50"/>
+      <c r="E15" s="50"/>
+      <c r="F15" s="50"/>
+      <c r="G15" s="50"/>
+      <c r="H15" s="50"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="50" t="str">
+        <v>Requêtes externes : aucune consultation distincte du tri. Les comparaisons et appels récursifs sont internes au traitement.</v>
+      </c>
+      <c r="B16" s="50"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="50"/>
+      <c r="F16" s="50"/>
+      <c r="G16" s="50"/>
+      <c r="H16" s="50"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="50" t="str">
+        <v>Fichiers internes et externes : aucun fichier ni groupe de données persistant dans le code étudié. Le tableau est en mémoire.</v>
+      </c>
+      <c r="B17" s="50"/>
+      <c r="C17" s="50"/>
+      <c r="D17" s="50"/>
+      <c r="E17" s="50"/>
+      <c r="F17" s="50"/>
+      <c r="G17" s="50"/>
+      <c r="H17" s="50"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="50" t="str">
+        <v>Niveau simple retenu pour les échanges : une liste d’entiers et sa taille, sans format complexe. Ce choix ne mesure pas la difficulté du tri.</v>
+      </c>
+      <c r="B18" s="50"/>
+      <c r="C18" s="50"/>
+      <c r="D18" s="50"/>
+      <c r="E18" s="50"/>
+      <c r="F18" s="50"/>
+      <c r="G18" s="50"/>
+      <c r="H18" s="50"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="50" t="str">
+        <v>Cette adaptation suppose que le tableau trié compte comme sortie du service. Ce n’est pas un décompte normalisé établi par le CM.</v>
+      </c>
+      <c r="B19" s="50"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
+      <c r="F19" s="50"/>
+      <c r="G19" s="50"/>
+      <c r="H19" s="50"/>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="50" t="str">
+        <v>Les poids sont conservés du CM ; les scores de son exemple sont remplacés par les nombres d’interactions retenus pour QuickSort.</v>
+      </c>
+      <c r="B20" s="50"/>
+      <c r="C20" s="50"/>
+      <c r="D20" s="50"/>
+      <c r="E20" s="50"/>
+      <c r="F20" s="50"/>
+      <c r="G20" s="50"/>
+      <c r="H20" s="50"/>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="50" t="str">
+        <v>Sources : CM R5.A.08, « Méthode des points de fonction d’Albrecht », p. 46 ; TP Mesures logicielles, exercice 2, Q4 et Q9.</v>
+      </c>
+      <c r="B21" s="50"/>
+      <c r="C21" s="50"/>
+      <c r="D21" s="50"/>
+      <c r="E21" s="50"/>
+      <c r="F21" s="50"/>
+      <c r="G21" s="50"/>
+      <c r="H21" s="50"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A13:H13"/>
+    <mergeCell ref="A14:H14"/>
+    <mergeCell ref="A15:H15"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A17:H17"/>
+    <mergeCell ref="A18:H18"/>
+    <mergeCell ref="A19:H19"/>
+    <mergeCell ref="A20:H20"/>
+    <mergeCell ref="A21:H21"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
MI avec les lignes de code
</commit_message>
<xml_diff>
--- a/fiche_de_calcul.xlsx
+++ b/fiche_de_calcul.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="5"/>
+    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
     <sheet name="Halstead" sheetId="1" state="visible" r:id="rId3"/>
@@ -14,6 +14,7 @@
     <sheet name="UFC-Q8" sheetId="4" state="visible" r:id="rId6"/>
     <sheet name="UFC-Q9" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="MI-Q10" sheetId="6" state="visible" r:id="rId8"/>
+    <sheet name="MI-Q11" sheetId="7" state="visible" r:id="rId9"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="99" uniqueCount="74">
   <si>
     <t xml:space="preserve">Opérateurs</t>
   </si>
@@ -295,6 +296,9 @@
   </si>
   <si>
     <t xml:space="preserve">MI</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LOC </t>
   </si>
 </sst>
 </file>
@@ -479,109 +483,117 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="165" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="13" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -834,251 +846,251 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:E22"/>
-  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="31.33"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="33.5"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="31.33"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="33.51"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="0" t="s">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="0" t="n">
+      <c r="E2" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E3" s="0" t="n">
+      <c r="E3" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="0" t="n">
+      <c r="E4" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D5" s="1" t="s">
+      <c r="D5" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="0" t="n">
+      <c r="E5" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>1</v>
       </c>
-      <c r="D6" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="E6" s="0" t="n">
+      <c r="D6" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D7" s="1" t="n">
+      <c r="D7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="E7" s="0" t="n">
+      <c r="E7" s="1" t="n">
         <v>4</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="0" t="n">
+      <c r="B8" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D8" s="1" t="s">
+      <c r="D8" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="E8" s="0" t="n">
+      <c r="E8" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="0" t="n">
+      <c r="B9" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D9" s="1" t="s">
+      <c r="D9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="E9" s="0" t="n">
+      <c r="E9" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="0" t="n">
+      <c r="B10" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="0" t="n">
+      <c r="B11" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="1" t="n">
+      <c r="B12" s="2" t="n">
         <f aca="false">SUM(B2:B11)</f>
         <v>16</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D12" s="1" t="n">
+      <c r="D12" s="2" t="n">
         <f aca="false">ROWS(D2:D9)</f>
         <v>8</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+      <c r="A13" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="2" t="s">
+      <c r="A14" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="1" t="n">
+      <c r="B14" s="2" t="n">
         <f aca="false">ROWS(B2:B11)</f>
         <v>10</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="D14" s="1" t="n">
+      <c r="D14" s="2" t="n">
         <f aca="false">SUM(E2:E9)</f>
         <v>35</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C15" s="0" t="s">
+      <c r="C15" s="1" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="B17" s="0" t="s">
+      <c r="B17" s="1" t="s">
         <v>28</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="B18" s="0" t="n">
+      <c r="B18" s="1" t="n">
         <f aca="false">B12+D14</f>
         <v>51</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="B19" s="0" t="n">
+      <c r="B19" s="1" t="n">
         <f aca="false">B14+D12</f>
         <v>18</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="17.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="B20" s="0" t="n">
+      <c r="B20" s="1" t="n">
         <f aca="false">B18*LOG(B19,2)</f>
         <v>212.666175073558</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="B21" s="0" t="n">
+      <c r="B21" s="1" t="n">
         <f aca="false">(B14/2)*(D14/D12)</f>
         <v>21.875</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="B22" s="0" t="n">
+      <c r="B22" s="1" t="n">
         <f aca="false">B21*B20</f>
         <v>4652.07257973408</v>
       </c>
@@ -1100,13 +1112,13 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:B1"/>
-  <sheetFormatPr defaultColWidth="10.50390625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="10.5078125" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
     <row r="1" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="0" t="n">
+      <c r="B1" s="1" t="n">
         <v>920</v>
       </c>
     </row>
@@ -1127,320 +1139,320 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:G33"/>
-  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="23.83"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="23.83"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="13"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="27" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="7" t="s">
+      <c r="A2" s="8" t="s">
         <v>37</v>
       </c>
-      <c r="B2" s="8" t="n">
+      <c r="B2" s="9" t="n">
         <v>12</v>
       </c>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
     </row>
     <row r="3" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="9" t="s">
+      <c r="A3" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="B3" s="8" t="n">
+      <c r="B3" s="9" t="n">
         <v>14</v>
       </c>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
     </row>
     <row r="4" customFormat="false" ht="34.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="11" t="s">
         <v>39</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="9" t="n">
         <f aca="false">B3 - B2 + 2</f>
         <v>4</v>
       </c>
-      <c r="C4" s="8"/>
-      <c r="D4" s="8"/>
-      <c r="E4" s="8"/>
-      <c r="F4" s="8"/>
-      <c r="G4" s="8"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="11"/>
-      <c r="B5" s="8"/>
-      <c r="C5" s="8"/>
-      <c r="D5" s="8"/>
-      <c r="E5" s="8"/>
-      <c r="F5" s="8"/>
-      <c r="G5" s="8"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="11"/>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8"/>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8"/>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
+      <c r="A6" s="12"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="9"/>
+      <c r="D6" s="9"/>
+      <c r="E6" s="9"/>
+      <c r="F6" s="9"/>
+      <c r="G6" s="9"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="11"/>
-      <c r="B7" s="8"/>
-      <c r="C7" s="8"/>
-      <c r="D7" s="8"/>
-      <c r="E7" s="8"/>
-      <c r="F7" s="8"/>
-      <c r="G7" s="8"/>
+      <c r="A7" s="12"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="9"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11"/>
-      <c r="B8" s="8"/>
-      <c r="C8" s="8"/>
-      <c r="D8" s="8"/>
-      <c r="E8" s="8"/>
-      <c r="F8" s="8"/>
-      <c r="G8" s="8"/>
+      <c r="A8" s="12"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="11"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="A9" s="12"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="11"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="A10" s="12"/>
+      <c r="B10" s="9"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="11"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="A11" s="12"/>
+      <c r="B11" s="9"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="11"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="A12" s="12"/>
+      <c r="B12" s="9"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
     </row>
     <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="11"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="A13" s="12"/>
+      <c r="B13" s="9"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
     </row>
     <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="11"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="A14" s="12"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
     </row>
     <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="A15" s="12"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
     </row>
     <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="11"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="A16" s="12"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="9"/>
+      <c r="D16" s="9"/>
+      <c r="E16" s="9"/>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
     </row>
     <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="11"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="A17" s="12"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="9"/>
+      <c r="D17" s="9"/>
+      <c r="E17" s="9"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
     </row>
     <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
+      <c r="A18" s="12"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="9"/>
+      <c r="D18" s="9"/>
+      <c r="E18" s="9"/>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
     </row>
     <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="11"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="A19" s="12"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="9"/>
+      <c r="D19" s="9"/>
+      <c r="E19" s="9"/>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
     </row>
     <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="11"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
+      <c r="A20" s="12"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="9"/>
+      <c r="D20" s="9"/>
+      <c r="E20" s="9"/>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
     </row>
     <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
+      <c r="A21" s="12"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="9"/>
+      <c r="D21" s="9"/>
+      <c r="E21" s="9"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
     </row>
     <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+      <c r="A22" s="9"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="9"/>
+      <c r="D22" s="9"/>
+      <c r="E22" s="9"/>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
     </row>
     <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="A23" s="9"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="9"/>
+      <c r="D23" s="9"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
     </row>
     <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+      <c r="A24" s="9"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="9"/>
+      <c r="D24" s="9"/>
+      <c r="E24" s="9"/>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
     </row>
     <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+      <c r="A25" s="9"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="9"/>
+      <c r="D25" s="9"/>
+      <c r="E25" s="9"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
     </row>
     <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+      <c r="A26" s="9"/>
+      <c r="B26" s="9"/>
+      <c r="C26" s="9"/>
+      <c r="D26" s="9"/>
+      <c r="E26" s="9"/>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
     </row>
     <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+      <c r="A27" s="9"/>
+      <c r="B27" s="9"/>
+      <c r="C27" s="9"/>
+      <c r="D27" s="9"/>
+      <c r="E27" s="9"/>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
     </row>
     <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
+      <c r="A28" s="9"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="9"/>
+      <c r="D28" s="9"/>
+      <c r="E28" s="9"/>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
     </row>
     <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
+      <c r="A29" s="9"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="9"/>
+      <c r="D29" s="9"/>
+      <c r="E29" s="9"/>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
     </row>
     <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
+      <c r="A30" s="9"/>
+      <c r="B30" s="9"/>
+      <c r="C30" s="9"/>
+      <c r="D30" s="9"/>
+      <c r="E30" s="9"/>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
     </row>
     <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
+      <c r="A31" s="9"/>
+      <c r="B31" s="9"/>
+      <c r="C31" s="9"/>
+      <c r="D31" s="9"/>
+      <c r="E31" s="9"/>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
     </row>
     <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="8"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
+      <c r="A32" s="9"/>
+      <c r="B32" s="9"/>
+      <c r="C32" s="9"/>
+      <c r="D32" s="9"/>
+      <c r="E32" s="9"/>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
     </row>
     <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="8"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
+      <c r="A33" s="9"/>
+      <c r="B33" s="9"/>
+      <c r="C33" s="9"/>
+      <c r="D33" s="9"/>
+      <c r="E33" s="9"/>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
     </row>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
@@ -1459,204 +1471,204 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:D21"/>
-  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.6640625" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.67"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="17.67"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="13" t="s">
         <v>40</v>
       </c>
-      <c r="B1" s="12"/>
+      <c r="B1" s="13"/>
     </row>
     <row r="2" customFormat="false" ht="20.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="14" t="s">
+      <c r="C2" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D2" s="14" t="s">
+      <c r="D2" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="15" t="s">
+      <c r="A3" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C3" s="0" t="n">
+      <c r="C3" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D3" s="0" t="n">
+      <c r="D3" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="15" t="s">
+      <c r="A4" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C4" s="0" t="n">
+      <c r="C4" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D4" s="0" t="n">
+      <c r="D4" s="1" t="n">
         <v>7</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="15" t="s">
+      <c r="A5" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B5" s="0" t="n">
+      <c r="B5" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="0" t="n">
+      <c r="C5" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="0" t="n">
+      <c r="D5" s="1" t="n">
         <v>6</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="15" t="s">
+      <c r="A6" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B6" s="0" t="n">
+      <c r="B6" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C6" s="0" t="n">
+      <c r="C6" s="1" t="n">
         <v>10</v>
       </c>
-      <c r="D6" s="0" t="n">
+      <c r="D6" s="1" t="n">
         <v>15</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="15" t="s">
+      <c r="A7" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="C7" s="0" t="n">
+      <c r="C7" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="D7" s="0" t="n">
+      <c r="D7" s="1" t="n">
         <v>10</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="13" t="s">
         <v>50</v>
       </c>
-      <c r="B10" s="12"/>
+      <c r="B10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="13" t="s">
+      <c r="A11" s="14" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="14" t="s">
+      <c r="B11" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="14" t="s">
+      <c r="D11" s="15" t="s">
         <v>44</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="15" t="s">
+      <c r="A12" s="16" t="s">
         <v>45</v>
       </c>
-      <c r="B12" s="0" t="n">
+      <c r="B12" s="1" t="n">
         <v>4</v>
       </c>
-      <c r="C12" s="0" t="n">
+      <c r="C12" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="D12" s="0" t="n">
+      <c r="D12" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="15" t="s">
+      <c r="A13" s="16" t="s">
         <v>46</v>
       </c>
-      <c r="B13" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="0" t="n">
+      <c r="B13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C13" s="1" t="n">
         <v>2</v>
       </c>
-      <c r="D13" s="0" t="n">
+      <c r="D13" s="1" t="n">
         <v>1</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="15" t="s">
+      <c r="A14" s="16" t="s">
         <v>47</v>
       </c>
-      <c r="B14" s="0" t="n">
+      <c r="B14" s="1" t="n">
         <v>7</v>
       </c>
-      <c r="C14" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D14" s="0" t="n">
+      <c r="C14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="15" t="s">
+      <c r="A15" s="16" t="s">
         <v>48</v>
       </c>
-      <c r="B15" s="0" t="n">
+      <c r="B15" s="1" t="n">
         <v>3</v>
       </c>
-      <c r="C15" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="D15" s="0" t="n">
+      <c r="C15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>49</v>
       </c>
-      <c r="B16" s="0" t="n">
-        <v>0</v>
-      </c>
-      <c r="C16" s="0" t="n">
+      <c r="B16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="C16" s="1" t="n">
         <v>5</v>
       </c>
-      <c r="D16" s="0" t="n">
+      <c r="D16" s="1" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="8.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="16"/>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
-      <c r="D17" s="16"/>
+      <c r="A17" s="17"/>
+      <c r="B17" s="17"/>
+      <c r="C17" s="17"/>
+      <c r="D17" s="17"/>
     </row>
     <row r="18" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="19" customFormat="false" ht="7.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
     <row r="20" customFormat="false" ht="33" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="17" t="s">
+      <c r="A20" s="18" t="s">
         <v>51</v>
       </c>
-      <c r="B20" s="4" t="n">
+      <c r="B20" s="5" t="n">
         <f aca="false">SUMPRODUCT(B3:D7,B12:D16)</f>
         <v>144</v>
       </c>
@@ -1683,353 +1695,353 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:H21"/>
-  <sheetFormatPr defaultColWidth="8.83203125" defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.8359375" defaultRowHeight="15.75" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="26"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="2" style="1" width="14"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>52</v>
       </c>
-      <c r="B1" s="19"/>
-      <c r="C1" s="19"/>
-      <c r="D1" s="19"/>
-      <c r="E1" s="19"/>
-      <c r="F1" s="19"/>
-      <c r="G1" s="19"/>
-      <c r="H1" s="19"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19"/>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
+      <c r="G2" s="20"/>
+      <c r="H2" s="20"/>
     </row>
     <row r="3" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20" t="s">
+      <c r="A3" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="21" t="s">
         <v>53</v>
       </c>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20" t="s">
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+      <c r="E3" s="21" t="s">
         <v>54</v>
       </c>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20" t="s">
+      <c r="F3" s="21"/>
+      <c r="G3" s="21"/>
+      <c r="H3" s="21" t="s">
         <v>55</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20"/>
-      <c r="B4" s="20" t="s">
+      <c r="A4" s="21"/>
+      <c r="B4" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="C4" s="20" t="s">
+      <c r="C4" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="D4" s="20" t="s">
+      <c r="D4" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="E4" s="20" t="s">
+      <c r="E4" s="21" t="s">
         <v>42</v>
       </c>
-      <c r="F4" s="20" t="s">
+      <c r="F4" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="G4" s="20" t="s">
+      <c r="G4" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="H4" s="20"/>
+      <c r="H4" s="21"/>
     </row>
     <row r="5" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="19" t="s">
+      <c r="A5" s="20" t="s">
         <v>45</v>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="E5" s="22" t="n">
+      <c r="E5" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="F5" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G5" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" s="21" t="n">
+      <c r="F5" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" s="22" t="n">
         <f aca="false">B5*E5+C5*F5+D5*G5</f>
         <v>3</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="19" t="s">
+      <c r="A6" s="20" t="s">
         <v>46</v>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="E6" s="22" t="n">
+      <c r="E6" s="23" t="n">
         <v>1</v>
       </c>
-      <c r="F6" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G6" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H6" s="21" t="n">
+      <c r="F6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="22" t="n">
         <f aca="false">B6*E6+C6*F6+D6*G6</f>
         <v>4</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="19" t="s">
+      <c r="A7" s="20" t="s">
         <v>56</v>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="E7" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G7" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H7" s="21" t="n">
+      <c r="E7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="22" t="n">
         <f aca="false">B7*E7+C7*F7+D7*G7</f>
         <v>0</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="19" t="s">
+      <c r="A8" s="20" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="21" t="n">
+      <c r="B8" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="E8" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F8" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G8" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H8" s="21" t="n">
+      <c r="E8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="22" t="n">
         <f aca="false">B8*E8+C8*F8+D8*G8</f>
         <v>0</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="19" t="s">
+      <c r="A9" s="20" t="s">
         <v>49</v>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="E9" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="F9" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="G9" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="H9" s="21" t="n">
+      <c r="E9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="22" t="n">
         <f aca="false">B9*E9+C9*F9+D9*G9</f>
         <v>0</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+      <c r="A10" s="21" t="s">
         <v>57</v>
       </c>
-      <c r="B10" s="23"/>
-      <c r="C10" s="23"/>
-      <c r="D10" s="23"/>
-      <c r="E10" s="23"/>
-      <c r="F10" s="23"/>
-      <c r="G10" s="23"/>
-      <c r="H10" s="23" t="n">
+      <c r="B10" s="24"/>
+      <c r="C10" s="24"/>
+      <c r="D10" s="24"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="24"/>
+      <c r="H10" s="24" t="n">
         <f aca="false">SUM(H5:H9)</f>
         <v>7</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="19"/>
-      <c r="B11" s="19"/>
-      <c r="C11" s="19"/>
-      <c r="D11" s="19"/>
-      <c r="E11" s="19"/>
-      <c r="F11" s="19"/>
-      <c r="G11" s="19"/>
-      <c r="H11" s="19"/>
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
     </row>
     <row r="12" customFormat="false" ht="24" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="24" t="s">
+      <c r="A12" s="25" t="s">
         <v>58</v>
       </c>
-      <c r="B12" s="19"/>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19"/>
-      <c r="E12" s="19"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="19"/>
-      <c r="H12" s="19"/>
+      <c r="B12" s="20"/>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="20"/>
     </row>
     <row r="13" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="25" t="s">
+      <c r="A13" s="26" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25"/>
-      <c r="F13" s="25"/>
-      <c r="G13" s="25"/>
-      <c r="H13" s="25"/>
+      <c r="B13" s="26"/>
+      <c r="C13" s="26"/>
+      <c r="D13" s="26"/>
+      <c r="E13" s="26"/>
+      <c r="F13" s="26"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="26"/>
     </row>
     <row r="14" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="25" t="s">
+      <c r="A14" s="26" t="s">
         <v>60</v>
       </c>
-      <c r="B14" s="25"/>
-      <c r="C14" s="25"/>
-      <c r="D14" s="25"/>
-      <c r="E14" s="25"/>
-      <c r="F14" s="25"/>
-      <c r="G14" s="25"/>
-      <c r="H14" s="25"/>
+      <c r="B14" s="26"/>
+      <c r="C14" s="26"/>
+      <c r="D14" s="26"/>
+      <c r="E14" s="26"/>
+      <c r="F14" s="26"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="26"/>
     </row>
     <row r="15" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="25" t="s">
+      <c r="A15" s="26" t="s">
         <v>61</v>
       </c>
-      <c r="B15" s="25"/>
-      <c r="C15" s="25"/>
-      <c r="D15" s="25"/>
-      <c r="E15" s="25"/>
-      <c r="F15" s="25"/>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
+      <c r="B15" s="26"/>
+      <c r="C15" s="26"/>
+      <c r="D15" s="26"/>
+      <c r="E15" s="26"/>
+      <c r="F15" s="26"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="26"/>
     </row>
     <row r="16" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="25" t="s">
+      <c r="A16" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
-      <c r="F16" s="25"/>
-      <c r="G16" s="25"/>
-      <c r="H16" s="25"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="25" t="s">
+      <c r="A17" s="26" t="s">
         <v>63</v>
       </c>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
     </row>
     <row r="18" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="25" t="s">
+      <c r="A18" s="26" t="s">
         <v>64</v>
       </c>
-      <c r="B18" s="25"/>
-      <c r="C18" s="25"/>
-      <c r="D18" s="25"/>
-      <c r="E18" s="25"/>
-      <c r="F18" s="25"/>
-      <c r="G18" s="25"/>
-      <c r="H18" s="25"/>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
+      <c r="D18" s="26"/>
+      <c r="E18" s="26"/>
+      <c r="F18" s="26"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="26"/>
     </row>
     <row r="19" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="25" t="s">
+      <c r="A19" s="26" t="s">
         <v>65</v>
       </c>
-      <c r="B19" s="25"/>
-      <c r="C19" s="25"/>
-      <c r="D19" s="25"/>
-      <c r="E19" s="25"/>
-      <c r="F19" s="25"/>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="26"/>
     </row>
     <row r="20" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="25" t="s">
+      <c r="A20" s="26" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="25"/>
-      <c r="C20" s="25"/>
-      <c r="D20" s="25"/>
-      <c r="E20" s="25"/>
-      <c r="F20" s="25"/>
-      <c r="G20" s="25"/>
-      <c r="H20" s="25"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
+      <c r="D20" s="26"/>
+      <c r="E20" s="26"/>
+      <c r="F20" s="26"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="26"/>
     </row>
     <row r="21" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="25" t="s">
+      <c r="A21" s="26" t="s">
         <v>67</v>
       </c>
-      <c r="B21" s="25"/>
-      <c r="C21" s="25"/>
-      <c r="D21" s="25"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="25"/>
-      <c r="G21" s="25"/>
-      <c r="H21" s="25"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
+      <c r="D21" s="26"/>
+      <c r="E21" s="26"/>
+      <c r="F21" s="26"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="9">
@@ -2058,50 +2070,124 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:B7"/>
-  <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <sheetData>
-    <row r="2" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="B2" s="0" t="n">
+      <c r="B2" s="1" t="n">
         <f aca="false">Halstead!B20</f>
         <v>212.666175073558</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="B3" s="0" t="n">
+      <c r="B3" s="1" t="n">
         <v>12</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="B4" s="0" t="n">
+      <c r="B4" s="1" t="n">
         <f aca="false">CC!B4</f>
         <v>4</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="B5" s="0" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="B5" s="1" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
         <v>72</v>
       </c>
-      <c r="B7" s="0" t="n">
+      <c r="B7" s="1" t="n">
         <f aca="false">171 - 5.2*LN(B2) - 0.23*B4 - 16.2*LN(B3) + 50*SIN(SQRT(2.46 * B5))</f>
         <v>101.953949121275</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,Normal"&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;KffffffPage &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:B7"/>
+  <sheetFormatPr defaultColWidth="9.34375" defaultRowHeight="12.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.37"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="10.37"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
+        <v>68</v>
+      </c>
+      <c r="B2" s="1" t="n">
+        <f aca="false">Halstead!B20</f>
+        <v>212.666175073558</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="18.7" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="B3" s="1" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="17" t="s">
+        <v>70</v>
+      </c>
+      <c r="B4" s="1" t="n">
+        <f aca="false">CC!B4</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="17" t="s">
+        <v>71</v>
+      </c>
+      <c r="B5" s="1" t="n">
+        <f aca="false"> (10/12)*100</f>
+        <v>83.3333333333333</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="27"/>
+      <c r="B6" s="1"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="17" t="s">
+        <v>72</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <f aca="false">171 - 5.2*LN(B2) - 0.23*B4 - 16.2*LN(B3) + 50*SIN(SQRT(2.46 * B5))</f>
+        <v>151.140267876801</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Question 12 : calcul du TFC de Qalculate
</commit_message>
<xml_diff>
--- a/fiche_de_calcul.xlsx
+++ b/fiche_de_calcul.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ns2="http://schemas.libreoffice.org/">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -8,18 +8,19 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="6"/>
   </bookViews>
   <sheets>
-    <sheet name="Halstead" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="LOC-Q6" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="CC" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="UFC-Q8" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="UFC-Q9" sheetId="5" state="visible" r:id="rId7"/>
-    <sheet name="MI-Q10" sheetId="6" state="visible" r:id="rId8"/>
-    <sheet name="MI-Q11" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Halstead" sheetId="1" state="visible" ns1:id="rId3"/>
+    <sheet name="LOC-Q6" sheetId="2" state="visible" ns1:id="rId4"/>
+    <sheet name="CC" sheetId="3" state="visible" ns1:id="rId5"/>
+    <sheet name="UFC-Q8" sheetId="4" state="visible" ns1:id="rId6"/>
+    <sheet name="UFC-Q9" sheetId="5" state="visible" ns1:id="rId7"/>
+    <sheet name="MI-Q10" sheetId="6" state="visible" ns1:id="rId8"/>
+    <sheet name="MI-Q11" sheetId="7" state="visible" ns1:id="rId9"/>
+    <sheet name="TFC-Q12" sheetId="8" ns1:id="rIdQ12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="ExcelA1"/>
+    <ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <ns2:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -305,11 +306,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0"/>
+    <numFmt numFmtId="166" formatCode="0"/>
+    <numFmt numFmtId="167" formatCode="0.00"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="31">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -407,8 +410,115 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <vertAlign val="subscript"/>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="13"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="20"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Carlito"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -427,8 +537,40 @@
         <bgColor rgb="FFE7E6E6"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="none"/>
+    </fill>
+    <fill>
+      <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE7E6E6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFF2CC"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="9">
     <border diagonalUp="false" diagonalDown="false">
       <left/>
       <right/>
@@ -457,6 +599,43 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="20">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
@@ -483,7 +662,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="69">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -595,6 +774,105 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0"/>
+    <xf numFmtId="0" fontId="20" fillId="4" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="4" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="4" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="4" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="4" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="4" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="4" borderId="4" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="24" fillId="4" borderId="4" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="24" fillId="6" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="24" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="1" fontId="23" fillId="4" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="1" fontId="23" fillId="7" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="25" fillId="4" borderId="4" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="26" fillId="8" borderId="8" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="28" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="11" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="27" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="8" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="27" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="30" fillId="10" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2199,4 +2477,420 @@
     <oddFooter>&amp;C&amp;"Times New Roman,Normal"&amp;KffffffPage &amp;P</oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="39" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="12" hidden="0" customWidth="1"/>
+    <col min="4" max="4" width="72" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="47" hidden="0" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="57" t="str">
+        <v>Q12 - Facteur de complexité technique de Qalculate!</v>
+      </c>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
+      <c r="E1" s="58"/>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="58" t="str">
+        <v>Périmètre : application de bureau Qalculate! (interface GTK et moteur libqalculate), calculs, définitions et taux de change.</v>
+      </c>
+      <c r="B2" s="58"/>
+      <c r="C2" s="58"/>
+      <c r="D2" s="58"/>
+      <c r="E2" s="58"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="58" t="str">
+        <v>Évaluation documentaire au 08/10/2026. Les scores sont des estimations argumentées, pas des mesures ni des notes officielles du projet.</v>
+      </c>
+      <c r="B3" s="58"/>
+      <c r="C3" s="58"/>
+      <c r="D3" s="58"/>
+      <c r="E3" s="58"/>
+    </row>
+    <row r="4" ht="30" customHeight="1">
+      <c r="A4" s="58" t="str">
+        <v>Échelle du CM : 0 = aucune influence ; 5 = influence critique. Convention retenue : 1 faible, 2 modérée, 3 moyenne, 4 forte.</v>
+      </c>
+      <c r="B4" s="58"/>
+      <c r="C4" s="58"/>
+      <c r="D4" s="58"/>
+      <c r="E4" s="58"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="58" t="str">
+        <v>« En ligne » = interaction pendant l’utilisation. Fichiers maîtres : définitions persistantes prises comme données de référence.</v>
+      </c>
+      <c r="B5" s="58"/>
+      <c r="C5" s="58"/>
+      <c r="D5" s="58"/>
+      <c r="E5" s="58"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="58"/>
+      <c r="B6" s="58"/>
+      <c r="C6" s="58"/>
+      <c r="D6" s="58"/>
+      <c r="E6" s="58"/>
+    </row>
+    <row r="7" ht="32" customHeight="1">
+      <c r="A7" s="62" t="str">
+        <v>N°</v>
+      </c>
+      <c r="B7" s="62" t="str">
+        <v>Facteur technique du CM</v>
+      </c>
+      <c r="C7" s="62" t="str">
+        <v>Note / 5</v>
+      </c>
+      <c r="D7" s="62" t="str">
+        <v>Justification et hypothèses</v>
+      </c>
+      <c r="E7" s="62" t="str">
+        <v>Source officielle</v>
+      </c>
+    </row>
+    <row r="8" ht="68" customHeight="1">
+      <c r="A8" s="59" t="n">
+        <v>1</v>
+      </c>
+      <c r="B8" s="59" t="str">
+        <v>Sauvegarde et récupération fiables</v>
+      </c>
+      <c r="C8" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D8" s="59" t="str">
+        <v>Historique et définitions conservés. Besoin modéré de préservation, sans exigence de reprise critique retenue.</v>
+      </c>
+      <c r="E8" s="60" t="str">
+        <v>https://qalculate.github.io/manual/qalculate-user-interface.html</v>
+      </c>
+    </row>
+    <row r="9" ht="68" customHeight="1">
+      <c r="A9" s="59" t="n">
+        <v>2</v>
+      </c>
+      <c r="B9" s="59" t="str">
+        <v>Communications de données</v>
+      </c>
+      <c r="C9" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D9" s="59" t="str">
+        <v>Téléchargement des taux de change. Influence limitée à cette fonction dans le périmètre étudié.</v>
+      </c>
+      <c r="E9" s="60" t="str">
+        <v>https://qalculate.github.io/manual/qalculate-units.html</v>
+      </c>
+    </row>
+    <row r="10" ht="68" customHeight="1">
+      <c r="A10" s="59" t="n">
+        <v>3</v>
+      </c>
+      <c r="B10" s="59" t="str">
+        <v>Traitement distribué</v>
+      </c>
+      <c r="C10" s="64" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="59" t="str">
+        <v>Calcul local retenu. Aucun traitement distribué documenté dans les fonctionnalités examinées ; télécharger des taux ne répartit pas le calcul.</v>
+      </c>
+      <c r="E10" s="60" t="str">
+        <v>https://github.com/Qalculate/qalculate-gtk</v>
+      </c>
+    </row>
+    <row r="11" ht="68" customHeight="1">
+      <c r="A11" s="59" t="n">
+        <v>4</v>
+      </c>
+      <c r="B11" s="59" t="str">
+        <v>Performances critiques</v>
+      </c>
+      <c r="C11" s="64" t="n">
+        <v>3</v>
+      </c>
+      <c r="D11" s="59" t="str">
+        <v>Le calcul au fil de la saisie motive une bonne réactivité. Influence moyenne, sans contrainte de temps réel critique supposée.</v>
+      </c>
+      <c r="E11" s="60" t="str">
+        <v>https://github.com/Qalculate/qalculate-gtk</v>
+      </c>
+    </row>
+    <row r="12" ht="68" customHeight="1">
+      <c r="A12" s="59" t="n">
+        <v>5</v>
+      </c>
+      <c r="B12" s="59" t="str">
+        <v>Environnement existant fortement utilisé</v>
+      </c>
+      <c r="C12" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D12" s="59" t="str">
+        <v>Hypothèse : poste de bureau ordinaire, partagé avec d’autres applications. Aucune forte contention démontrée ; faible influence retenue.</v>
+      </c>
+      <c r="E12" s="60" t="str">
+        <v>https://github.com/Qalculate/qalculate-gtk</v>
+      </c>
+    </row>
+    <row r="13" ht="68" customHeight="1">
+      <c r="A13" s="59" t="n">
+        <v>6</v>
+      </c>
+      <c r="B13" s="59" t="str">
+        <v>Entrées en ligne</v>
+      </c>
+      <c r="C13" s="64" t="n">
+        <v>4</v>
+      </c>
+      <c r="D13" s="59" t="str">
+        <v>La saisie interactive des expressions est le mode principal d’utilisation. Influence forte sur la conception de l’interface.</v>
+      </c>
+      <c r="E13" s="60" t="str">
+        <v>https://qalculate.github.io/manual/qalculate-user-interface.html</v>
+      </c>
+    </row>
+    <row r="14" ht="68" customHeight="1">
+      <c r="A14" s="59" t="n">
+        <v>7</v>
+      </c>
+      <c r="B14" s="59" t="str">
+        <v>Saisie sur plusieurs écrans</v>
+      </c>
+      <c r="C14" s="64" t="n">
+        <v>1</v>
+      </c>
+      <c r="D14" s="59" t="str">
+        <v>Le calcul courant tient dans la fenêtre principale. Des dialogues servent aux matrices ou fonctions ; influence faible.</v>
+      </c>
+      <c r="E14" s="60" t="str">
+        <v>https://qalculate.github.io/manual/qalculate-user-interface.html</v>
+      </c>
+    </row>
+    <row r="15" ht="68" customHeight="1">
+      <c r="A15" s="59" t="n">
+        <v>8</v>
+      </c>
+      <c r="B15" s="59" t="str">
+        <v>Mise à jour en ligne des fichiers maîtres</v>
+      </c>
+      <c r="C15" s="64" t="n">
+        <v>2</v>
+      </c>
+      <c r="D15" s="59" t="str">
+        <v>Les définitions personnelles peuvent être modifiées et sauvegardées. Assimilation pédagogique à des données de référence, sans base métier centrale.</v>
+      </c>
+      <c r="E15" s="60" t="str">
+        <v>https://qalculate.github.io/manual/qalculate-user-interface.html</v>
+      </c>
+    </row>
+    <row r="16" ht="68" customHeight="1">
+      <c r="A16" s="59" t="n">
+        <v>9</v>
+      </c>
+      <c r="B16" s="59" t="str">
+        <v>Complexité des entrées, sorties et fichiers</v>
+      </c>
+      <c r="C16" s="64" t="n">
+        <v>4</v>
+      </c>
+      <c r="D16" s="59" t="str">
+        <v>Expressions symboliques, unités et précision arbitraire imposent des représentations riches. Influence forte.</v>
+      </c>
+      <c r="E16" s="60" t="str">
+        <v>https://github.com/Qalculate/libqalculate</v>
+      </c>
+    </row>
+    <row r="17" ht="68" customHeight="1">
+      <c r="A17" s="59" t="n">
+        <v>10</v>
+      </c>
+      <c r="B17" s="59" t="str">
+        <v>Complexité du traitement interne</v>
+      </c>
+      <c r="C17" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D17" s="59" t="str">
+        <v>Calcul symbolique, équations, intégrales et propagation des incertitudes : traitements au cœur du produit. Influence critique retenue.</v>
+      </c>
+      <c r="E17" s="60" t="str">
+        <v>https://github.com/Qalculate/libqalculate</v>
+      </c>
+    </row>
+    <row r="18" ht="68" customHeight="1">
+      <c r="A18" s="59" t="n">
+        <v>11</v>
+      </c>
+      <c r="B18" s="59" t="str">
+        <v>Réutilisabilité du code</v>
+      </c>
+      <c r="C18" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D18" s="59" t="str">
+        <v>Le moteur libqalculate est une bibliothèque distincte, utilisée par plusieurs interfaces. La réutilisation structure l’architecture.</v>
+      </c>
+      <c r="E18" s="60" t="str">
+        <v>https://github.com/Qalculate/libqalculate</v>
+      </c>
+    </row>
+    <row r="19" ht="68" customHeight="1">
+      <c r="A19" s="59" t="n">
+        <v>12</v>
+      </c>
+      <c r="B19" s="59" t="str">
+        <v>Conversion et installation prévues</v>
+      </c>
+      <c r="C19" s="64" t="n">
+        <v>3</v>
+      </c>
+      <c r="D19" s="59" t="str">
+        <v>Installateurs, archives portables et paquets sont proposés. Installation prise en compte ; pas de migration métier complexe supposée.</v>
+      </c>
+      <c r="E19" s="60" t="str">
+        <v>https://qalculate.github.io/downloads.html</v>
+      </c>
+    </row>
+    <row r="20" ht="68" customHeight="1">
+      <c r="A20" s="59" t="n">
+        <v>13</v>
+      </c>
+      <c r="B20" s="59" t="str">
+        <v>Multiples organisations ou plateformes</v>
+      </c>
+      <c r="C20" s="64" t="n">
+        <v>4</v>
+      </c>
+      <c r="D20" s="59" t="str">
+        <v>Distribution pour Windows, macOS et GNU/Linux. La portabilité justifie une influence forte, sans supposer un système multi-organisations.</v>
+      </c>
+      <c r="E20" s="60" t="str">
+        <v>https://qalculate.github.io/downloads.html</v>
+      </c>
+    </row>
+    <row r="21" ht="68" customHeight="1">
+      <c r="A21" s="59" t="n">
+        <v>14</v>
+      </c>
+      <c r="B21" s="59" t="str">
+        <v>Facilité d’utilisation</v>
+      </c>
+      <c r="C21" s="64" t="n">
+        <v>5</v>
+      </c>
+      <c r="D21" s="59" t="str">
+        <v>Complétion, aide à la saisie et historique facilitent les calculs. L’ergonomie est retenue comme exigence centrale.</v>
+      </c>
+      <c r="E21" s="60" t="str">
+        <v>https://github.com/Qalculate/qalculate-gtk</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="58"/>
+      <c r="B22" s="58"/>
+      <c r="C22" s="65"/>
+      <c r="D22" s="58"/>
+      <c r="E22" s="58"/>
+    </row>
+    <row r="23" ht="28" customHeight="1">
+      <c r="A23" s="58"/>
+      <c r="B23" s="58" t="str">
+        <v>Somme des 14 notes</v>
+      </c>
+      <c r="C23" s="65" t="n">
+        <f>SUM(C8:C21)</f>
+        <v>41</v>
+      </c>
+      <c r="D23" s="58"/>
+      <c r="E23" s="58"/>
+    </row>
+    <row r="24" ht="28" customHeight="1">
+      <c r="A24" s="58"/>
+      <c r="B24" s="58" t="str">
+        <v>Constante du CM</v>
+      </c>
+      <c r="C24" s="66" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="D24" s="58"/>
+      <c r="E24" s="58"/>
+    </row>
+    <row r="25" ht="28" customHeight="1">
+      <c r="A25" s="58"/>
+      <c r="B25" s="58" t="str">
+        <v>Coefficient du CM</v>
+      </c>
+      <c r="C25" s="66" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="D25" s="58"/>
+      <c r="E25" s="58"/>
+    </row>
+    <row r="26" ht="28" customHeight="1">
+      <c r="A26" s="58"/>
+      <c r="B26" s="62" t="str">
+        <v>TFC = 0,65 + 0,01 × somme</v>
+      </c>
+      <c r="C26" s="68" t="n">
+        <f>C24+C25*C23</f>
+        <v>1.06</v>
+      </c>
+      <c r="D26" s="58"/>
+      <c r="E26" s="58"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="58"/>
+      <c r="B27" s="58"/>
+      <c r="C27" s="58"/>
+      <c r="D27" s="58"/>
+      <c r="E27" s="58"/>
+    </row>
+    <row r="28" ht="32" customHeight="1">
+      <c r="A28" s="58" t="str">
+        <v>Source de la méthode : CM R5.A.08, pages 47-48 (formule et ordre des 14 facteurs). Le TD écrit TFC ; le CM emploie TCF.</v>
+      </c>
+      <c r="B28" s="58"/>
+      <c r="C28" s="58"/>
+      <c r="D28" s="58"/>
+      <c r="E28" s="58"/>
+    </row>
+    <row r="29" ht="32" customHeight="1">
+      <c r="A29" s="58" t="str">
+        <v>Le facteur obtenu concerne Qalculate! : il ne doit pas être multiplié par l’UFC de QuickSort, qui décrit un autre système.</v>
+      </c>
+      <c r="B29" s="58"/>
+      <c r="C29" s="58"/>
+      <c r="D29" s="58"/>
+      <c r="E29" s="58"/>
+    </row>
+  </sheetData>
+  <mergeCells>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A5:E5"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A29:E29"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation type="whole" operator="between" sqref="C8:C21">
+      <formula1>0</formula1>
+      <formula2>5</formula2>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>